<commit_message>
New onset and coda map
</commit_message>
<xml_diff>
--- a/default_layout.xlsx
+++ b/default_layout.xlsx
@@ -55,33 +55,33 @@
     <t xml:space="preserve">ㅅ</t>
   </si>
   <si>
+    <t xml:space="preserve">ㅎ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㅇ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㄴ</t>
+  </si>
+  <si>
     <t xml:space="preserve">ㄹ</t>
   </si>
   <si>
-    <t xml:space="preserve">ㅇ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㄴ</t>
+    <t xml:space="preserve">ㅍ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㅊ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㅌ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㅋ</t>
   </si>
   <si>
     <t xml:space="preserve">ㅁ</t>
   </si>
   <si>
-    <t xml:space="preserve">ㅍ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㅊ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㅌ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㅋ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㅎ</t>
-  </si>
-  <si>
     <t xml:space="preserve">中聲</t>
   </si>
   <si>
@@ -151,37 +151,37 @@
     <t xml:space="preserve">終聲</t>
   </si>
   <si>
+    <t xml:space="preserve">ㄽ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㄺ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㄶ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㄼ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ㄿ</t>
+  </si>
+  <si>
     <t xml:space="preserve">ㄳ</t>
   </si>
   <si>
     <t xml:space="preserve">ㅀ</t>
   </si>
   <si>
-    <t xml:space="preserve">ㄶ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㄼ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㄿ</t>
-  </si>
-  <si>
     <t xml:space="preserve">ㅄ</t>
   </si>
   <si>
-    <t xml:space="preserve">ㄺ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㄽ</t>
-  </si>
-  <si>
     <t xml:space="preserve">ㄵ</t>
   </si>
   <si>
+    <t xml:space="preserve">ㄾ</t>
+  </si>
+  <si>
     <t xml:space="preserve">ㄻ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ㄾ</t>
   </si>
   <si>
     <t xml:space="preserve">QWERTY</t>
@@ -284,7 +284,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Noto Sans"/>
@@ -310,12 +310,18 @@
       <sz val="16"/>
       <name val="Source Han Sans CN"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="16"/>
       <name val="Noto Serif"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Source Han Sans CN"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="16"/>
@@ -379,7 +385,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -400,6 +406,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -408,7 +418,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -595,7 +605,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultColWidth="11.23046875" defaultRowHeight="14.35" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="1" width="5.52"/>
@@ -653,7 +663,7 @@
       <c r="E3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="5" t="s">
         <v>11</v>
       </c>
       <c r="G3" s="3" t="s">
@@ -662,7 +672,7 @@
       <c r="H3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="5" t="s">
         <v>14</v>
       </c>
       <c r="J3" s="4"/>
@@ -682,7 +692,7 @@
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="5" t="s">
         <v>19</v>
       </c>
       <c r="H4" s="4"/>
@@ -690,16 +700,16 @@
       <c r="J4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
@@ -794,16 +804,16 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="20.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
@@ -820,13 +830,13 @@
       <c r="J11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>3</v>
       </c>
       <c r="D12" s="3" t="s">
@@ -835,16 +845,16 @@
       <c r="E12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="5" t="s">
         <v>46</v>
       </c>
       <c r="J12" s="3" t="s">
@@ -867,8 +877,8 @@
       <c r="E13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>48</v>
+      <c r="F13" s="5" t="s">
+        <v>11</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>12</v>
@@ -876,11 +886,11 @@
       <c r="H13" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="3" t="s">
-        <v>11</v>
+      <c r="J13" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -896,137 +906,134 @@
       <c r="D14" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="J14" s="5" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="s">
+      <c r="A16" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+    </row>
+    <row r="17" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="J17" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+    <row r="18" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="J18" s="8" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
+    <row r="19" customFormat="false" ht="20.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="G19" s="7" t="s">
+      <c r="G19" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="H19" s="7" t="s">
+      <c r="H19" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="J19" s="7" t="s">
+      <c r="J19" s="8" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E22" s="0"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>